<commit_message>
Add the mandatory assignment page, remove the electricity workshop from the site
New page Mandatory_assignment.qmd (with a print-friendly PDF in pdfs/ and a
figure) in its own sidebar section. WS_electricityprices.qmd stays in the
folder but is excluded from the site render and removed from the sidebar.

The lab and assignment pages declare a pdf format, so html is now listed first
in their front matter; otherwise the sidebar links to the pdf instead of the
web page. Also updates lecturePlan.xlsx.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lecturePlan.xlsx
+++ b/lecturePlan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sondre/Documents/BAN430/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sondre/Library/CloudStorage/OneDrive-NorwegianSchoolofEconomics/Teaching/BAN430/BAN430_website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60BF5C6D-C4F2-884B-9EA4-D2465A89B79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{924C3464-85C5-C94F-A3DA-E1088742E600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="34560" windowHeight="19800" activeTab="3" xr2:uid="{DEDCCCE6-C2B3-4C3C-BD8B-2E3EEC4135F8}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="19800" activeTab="3" xr2:uid="{DEDCCCE6-C2B3-4C3C-BD8B-2E3EEC4135F8}"/>
   </bookViews>
   <sheets>
     <sheet name="kladd" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="131">
   <si>
     <t>Week number</t>
   </si>
@@ -426,6 +426,9 @@
   </si>
   <si>
     <t>Dynamic regression models</t>
+  </si>
+  <si>
+    <t>Do exercises/old exams</t>
   </si>
 </sst>
 </file>
@@ -2633,10 +2636,10 @@
     <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="85"/>
       <c r="B15" s="76" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C15" s="76" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -2653,10 +2656,10 @@
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="84"/>
       <c r="B17" s="48" t="s">
-        <v>43</v>
+        <v>129</v>
       </c>
       <c r="C17" s="48" t="s">
-        <v>43</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -2670,11 +2673,11 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="84"/>
-      <c r="B19" s="48" t="s">
-        <v>129</v>
-      </c>
-      <c r="C19" s="48" t="s">
-        <v>129</v>
+      <c r="B19" s="52" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="49" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -2688,11 +2691,11 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="84"/>
-      <c r="B21" s="52" t="s">
-        <v>95</v>
-      </c>
-      <c r="C21" s="49" t="s">
-        <v>95</v>
+      <c r="B21" s="53" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="53" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -2707,10 +2710,10 @@
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="84"/>
       <c r="B23" s="53" t="s">
-        <v>11</v>
+        <v>130</v>
       </c>
       <c r="C23" s="53" t="s">
-        <v>11</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>